<commit_message>
adding schawarma in cmd list
</commit_message>
<xml_diff>
--- a/cmdList.xlsx
+++ b/cmdList.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bianca\Desktop\Server biamine\custom plugin\1_Resourcepacks\Github\Ressourcepack-for-biamine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65A2DBDA-9730-4C9B-83F4-EEF8F2D4813E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933DC650-9A9E-4457-B3EF-5607A6396A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="167">
   <si>
     <t>Key (Legende)</t>
   </si>
@@ -518,6 +518,9 @@
   </si>
   <si>
     <t>brezel</t>
+  </si>
+  <si>
+    <t>schawarma</t>
   </si>
 </sst>
 </file>
@@ -1059,7 +1062,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J151"/>
+  <dimension ref="B2:J152"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -2085,40 +2088,40 @@
         <v>165</v>
       </c>
     </row>
-    <row r="78" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B78" s="23" t="s">
+    <row r="77" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B77" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C77" s="12">
+        <v>6</v>
+      </c>
+      <c r="D77" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E77" s="14" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="79" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B79" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="C78" s="24"/>
-      <c r="D78" s="24"/>
-      <c r="E78" s="24"/>
-    </row>
-    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B79" s="1" t="s">
+      <c r="C79" s="24"/>
+      <c r="D79" s="24"/>
+      <c r="E79" s="24"/>
+    </row>
+    <row r="80" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B80" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C79" s="1" t="s">
+      <c r="C80" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D79" s="1" t="s">
+      <c r="D80" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E79" s="2" t="s">
+      <c r="E80" s="2" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="80" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B80" s="12">
-        <v>1</v>
-      </c>
-      <c r="C80" s="12">
-        <v>1</v>
-      </c>
-      <c r="D80" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E80" s="14" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="81" spans="2:5" x14ac:dyDescent="0.25">
@@ -2129,10 +2132,10 @@
         <v>1</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E81" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="82" spans="2:5" x14ac:dyDescent="0.25">
@@ -2143,10 +2146,10 @@
         <v>1</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E82" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="83" spans="2:5" x14ac:dyDescent="0.25">
@@ -2157,118 +2160,118 @@
         <v>1</v>
       </c>
       <c r="D83" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E83" s="14" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="84" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B84" s="12">
+        <v>1</v>
+      </c>
+      <c r="C84" s="12">
+        <v>1</v>
+      </c>
+      <c r="D84" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E83" s="14" t="s">
+      <c r="E84" s="14" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="87" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B87" s="5"/>
-      <c r="C87" s="7" t="s">
+    <row r="88" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B88" s="5"/>
+      <c r="C88" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="D87" s="5"/>
-      <c r="E87" s="6"/>
-    </row>
-    <row r="89" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B89" s="25" t="s">
+      <c r="D88" s="5"/>
+      <c r="E88" s="6"/>
+    </row>
+    <row r="90" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B90" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="C89" s="24"/>
-      <c r="D89" s="24"/>
-      <c r="E89" s="24"/>
-    </row>
-    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B90" s="1" t="s">
+      <c r="C90" s="24"/>
+      <c r="D90" s="24"/>
+      <c r="E90" s="24"/>
+    </row>
+    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B91" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C90" s="1" t="s">
+      <c r="C91" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D90" s="9" t="s">
+      <c r="D91" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="E90" s="2" t="s">
+      <c r="E91" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B91" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C91" s="12">
-        <v>6</v>
-      </c>
-      <c r="D91" s="15" t="s">
+    <row r="92" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B92" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C92" s="12">
+        <v>6</v>
+      </c>
+      <c r="D92" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="E91" s="16" t="s">
+      <c r="E92" s="16" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="92" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B92" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="C92" s="17">
-        <v>6</v>
-      </c>
-      <c r="D92" s="18" t="s">
+    <row r="93" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B93" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C93" s="17">
+        <v>6</v>
+      </c>
+      <c r="D93" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="E92" s="19" t="s">
+      <c r="E93" s="19" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="94" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B94" s="25" t="s">
+    <row r="95" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B95" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="C94" s="24"/>
-      <c r="D94" s="24"/>
-      <c r="E94" s="24"/>
-    </row>
-    <row r="95" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B95" s="1" t="s">
+      <c r="C95" s="24"/>
+      <c r="D95" s="24"/>
+      <c r="E95" s="24"/>
+    </row>
+    <row r="96" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B96" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C95" s="1" t="s">
+      <c r="C96" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D95" s="9" t="s">
+      <c r="D96" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="E95" s="2" t="s">
+      <c r="E96" s="2" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="96" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B96" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C96" s="12">
-        <v>6</v>
-      </c>
-      <c r="D96" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E96" s="16" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="97" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B97" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C97" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="D97" s="18" t="s">
-        <v>105</v>
-      </c>
-      <c r="E97" s="21" t="s">
-        <v>104</v>
+      <c r="C97" s="12">
+        <v>6</v>
+      </c>
+      <c r="D97" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="E97" s="16" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="98" spans="2:5" x14ac:dyDescent="0.25">
@@ -2278,8 +2281,8 @@
       <c r="C98" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D98" s="15" t="s">
-        <v>106</v>
+      <c r="D98" s="18" t="s">
+        <v>105</v>
       </c>
       <c r="E98" s="21" t="s">
         <v>104</v>
@@ -2292,8 +2295,8 @@
       <c r="C99" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D99" s="22" t="s">
-        <v>107</v>
+      <c r="D99" s="15" t="s">
+        <v>106</v>
       </c>
       <c r="E99" s="21" t="s">
         <v>104</v>
@@ -2306,8 +2309,8 @@
       <c r="C100" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D100" s="15" t="s">
-        <v>108</v>
+      <c r="D100" s="22" t="s">
+        <v>107</v>
       </c>
       <c r="E100" s="21" t="s">
         <v>104</v>
@@ -2320,8 +2323,8 @@
       <c r="C101" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D101" s="18" t="s">
-        <v>105</v>
+      <c r="D101" s="15" t="s">
+        <v>108</v>
       </c>
       <c r="E101" s="21" t="s">
         <v>104</v>
@@ -2334,8 +2337,8 @@
       <c r="C102" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D102" s="15" t="s">
-        <v>109</v>
+      <c r="D102" s="18" t="s">
+        <v>105</v>
       </c>
       <c r="E102" s="21" t="s">
         <v>104</v>
@@ -2348,8 +2351,8 @@
       <c r="C103" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D103" s="18" t="s">
-        <v>110</v>
+      <c r="D103" s="15" t="s">
+        <v>109</v>
       </c>
       <c r="E103" s="21" t="s">
         <v>104</v>
@@ -2362,8 +2365,8 @@
       <c r="C104" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D104" s="15" t="s">
-        <v>111</v>
+      <c r="D104" s="18" t="s">
+        <v>110</v>
       </c>
       <c r="E104" s="21" t="s">
         <v>104</v>
@@ -2376,8 +2379,8 @@
       <c r="C105" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D105" s="22" t="s">
-        <v>112</v>
+      <c r="D105" s="15" t="s">
+        <v>111</v>
       </c>
       <c r="E105" s="21" t="s">
         <v>104</v>
@@ -2390,8 +2393,8 @@
       <c r="C106" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D106" s="15" t="s">
-        <v>113</v>
+      <c r="D106" s="22" t="s">
+        <v>112</v>
       </c>
       <c r="E106" s="21" t="s">
         <v>104</v>
@@ -2404,8 +2407,8 @@
       <c r="C107" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D107" s="22" t="s">
-        <v>114</v>
+      <c r="D107" s="15" t="s">
+        <v>113</v>
       </c>
       <c r="E107" s="21" t="s">
         <v>104</v>
@@ -2418,8 +2421,8 @@
       <c r="C108" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D108" s="15" t="s">
-        <v>115</v>
+      <c r="D108" s="22" t="s">
+        <v>114</v>
       </c>
       <c r="E108" s="21" t="s">
         <v>104</v>
@@ -2432,8 +2435,8 @@
       <c r="C109" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D109" s="18" t="s">
-        <v>116</v>
+      <c r="D109" s="15" t="s">
+        <v>115</v>
       </c>
       <c r="E109" s="21" t="s">
         <v>104</v>
@@ -2446,8 +2449,8 @@
       <c r="C110" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D110" s="15" t="s">
-        <v>117</v>
+      <c r="D110" s="18" t="s">
+        <v>116</v>
       </c>
       <c r="E110" s="21" t="s">
         <v>104</v>
@@ -2460,8 +2463,8 @@
       <c r="C111" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D111" s="18" t="s">
-        <v>118</v>
+      <c r="D111" s="15" t="s">
+        <v>117</v>
       </c>
       <c r="E111" s="21" t="s">
         <v>104</v>
@@ -2474,8 +2477,8 @@
       <c r="C112" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D112" s="15" t="s">
-        <v>119</v>
+      <c r="D112" s="18" t="s">
+        <v>118</v>
       </c>
       <c r="E112" s="21" t="s">
         <v>104</v>
@@ -2488,8 +2491,8 @@
       <c r="C113" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D113" s="18" t="s">
-        <v>120</v>
+      <c r="D113" s="15" t="s">
+        <v>119</v>
       </c>
       <c r="E113" s="21" t="s">
         <v>104</v>
@@ -2502,8 +2505,8 @@
       <c r="C114" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D114" s="15" t="s">
-        <v>121</v>
+      <c r="D114" s="18" t="s">
+        <v>120</v>
       </c>
       <c r="E114" s="21" t="s">
         <v>104</v>
@@ -2516,8 +2519,8 @@
       <c r="C115" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D115" s="18" t="s">
-        <v>122</v>
+      <c r="D115" s="15" t="s">
+        <v>121</v>
       </c>
       <c r="E115" s="21" t="s">
         <v>104</v>
@@ -2530,8 +2533,8 @@
       <c r="C116" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D116" s="15" t="s">
-        <v>123</v>
+      <c r="D116" s="18" t="s">
+        <v>122</v>
       </c>
       <c r="E116" s="21" t="s">
         <v>104</v>
@@ -2544,8 +2547,8 @@
       <c r="C117" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D117" s="18" t="s">
-        <v>124</v>
+      <c r="D117" s="15" t="s">
+        <v>123</v>
       </c>
       <c r="E117" s="21" t="s">
         <v>104</v>
@@ -2558,8 +2561,8 @@
       <c r="C118" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D118" s="15" t="s">
-        <v>125</v>
+      <c r="D118" s="18" t="s">
+        <v>124</v>
       </c>
       <c r="E118" s="21" t="s">
         <v>104</v>
@@ -2572,8 +2575,8 @@
       <c r="C119" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D119" s="18" t="s">
-        <v>126</v>
+      <c r="D119" s="15" t="s">
+        <v>125</v>
       </c>
       <c r="E119" s="21" t="s">
         <v>104</v>
@@ -2586,8 +2589,8 @@
       <c r="C120" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D120" s="15" t="s">
-        <v>127</v>
+      <c r="D120" s="18" t="s">
+        <v>126</v>
       </c>
       <c r="E120" s="21" t="s">
         <v>104</v>
@@ -2600,47 +2603,47 @@
       <c r="C121" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D121" s="18" t="s">
-        <v>128</v>
+      <c r="D121" s="15" t="s">
+        <v>127</v>
       </c>
       <c r="E121" s="21" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="123" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B123" s="25" t="s">
+    <row r="122" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B122" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C122" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D122" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="E122" s="21" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="124" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B124" s="25" t="s">
         <v>129</v>
       </c>
-      <c r="C123" s="24"/>
-      <c r="D123" s="24"/>
-      <c r="E123" s="24"/>
-    </row>
-    <row r="124" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B124" s="1" t="s">
+      <c r="C124" s="24"/>
+      <c r="D124" s="24"/>
+      <c r="E124" s="24"/>
+    </row>
+    <row r="125" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B125" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C124" s="1" t="s">
+      <c r="C125" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D124" s="9" t="s">
+      <c r="D125" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="E124" s="2" t="s">
+      <c r="E125" s="2" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="125" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B125" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C125" s="12">
-        <v>2</v>
-      </c>
-      <c r="D125" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="E125" s="16" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="126" spans="2:5" x14ac:dyDescent="0.25">
@@ -2650,8 +2653,8 @@
       <c r="C126" s="12">
         <v>2</v>
       </c>
-      <c r="D126" s="18" t="s">
-        <v>132</v>
+      <c r="D126" s="15" t="s">
+        <v>131</v>
       </c>
       <c r="E126" s="16" t="s">
         <v>130</v>
@@ -2664,8 +2667,8 @@
       <c r="C127" s="12">
         <v>2</v>
       </c>
-      <c r="D127" s="15" t="s">
-        <v>133</v>
+      <c r="D127" s="18" t="s">
+        <v>132</v>
       </c>
       <c r="E127" s="16" t="s">
         <v>130</v>
@@ -2678,8 +2681,8 @@
       <c r="C128" s="12">
         <v>2</v>
       </c>
-      <c r="D128" s="22" t="s">
-        <v>134</v>
+      <c r="D128" s="15" t="s">
+        <v>133</v>
       </c>
       <c r="E128" s="16" t="s">
         <v>130</v>
@@ -2692,8 +2695,8 @@
       <c r="C129" s="12">
         <v>2</v>
       </c>
-      <c r="D129" s="15" t="s">
-        <v>135</v>
+      <c r="D129" s="22" t="s">
+        <v>134</v>
       </c>
       <c r="E129" s="16" t="s">
         <v>130</v>
@@ -2706,8 +2709,8 @@
       <c r="C130" s="12">
         <v>2</v>
       </c>
-      <c r="D130" s="18" t="s">
-        <v>136</v>
+      <c r="D130" s="15" t="s">
+        <v>135</v>
       </c>
       <c r="E130" s="16" t="s">
         <v>130</v>
@@ -2720,8 +2723,8 @@
       <c r="C131" s="12">
         <v>2</v>
       </c>
-      <c r="D131" s="15" t="s">
-        <v>137</v>
+      <c r="D131" s="18" t="s">
+        <v>136</v>
       </c>
       <c r="E131" s="16" t="s">
         <v>130</v>
@@ -2734,8 +2737,8 @@
       <c r="C132" s="12">
         <v>2</v>
       </c>
-      <c r="D132" s="22" t="s">
-        <v>138</v>
+      <c r="D132" s="15" t="s">
+        <v>137</v>
       </c>
       <c r="E132" s="16" t="s">
         <v>130</v>
@@ -2748,8 +2751,8 @@
       <c r="C133" s="12">
         <v>2</v>
       </c>
-      <c r="D133" s="15" t="s">
-        <v>139</v>
+      <c r="D133" s="22" t="s">
+        <v>138</v>
       </c>
       <c r="E133" s="16" t="s">
         <v>130</v>
@@ -2762,8 +2765,8 @@
       <c r="C134" s="12">
         <v>2</v>
       </c>
-      <c r="D134" s="22" t="s">
-        <v>140</v>
+      <c r="D134" s="15" t="s">
+        <v>139</v>
       </c>
       <c r="E134" s="16" t="s">
         <v>130</v>
@@ -2776,8 +2779,8 @@
       <c r="C135" s="12">
         <v>2</v>
       </c>
-      <c r="D135" s="15" t="s">
-        <v>141</v>
+      <c r="D135" s="22" t="s">
+        <v>140</v>
       </c>
       <c r="E135" s="16" t="s">
         <v>130</v>
@@ -2790,8 +2793,8 @@
       <c r="C136" s="12">
         <v>2</v>
       </c>
-      <c r="D136" s="22" t="s">
-        <v>142</v>
+      <c r="D136" s="15" t="s">
+        <v>141</v>
       </c>
       <c r="E136" s="16" t="s">
         <v>130</v>
@@ -2804,8 +2807,8 @@
       <c r="C137" s="12">
         <v>2</v>
       </c>
-      <c r="D137" s="15" t="s">
-        <v>143</v>
+      <c r="D137" s="22" t="s">
+        <v>142</v>
       </c>
       <c r="E137" s="16" t="s">
         <v>130</v>
@@ -2818,8 +2821,8 @@
       <c r="C138" s="12">
         <v>2</v>
       </c>
-      <c r="D138" s="18" t="s">
-        <v>144</v>
+      <c r="D138" s="15" t="s">
+        <v>143</v>
       </c>
       <c r="E138" s="16" t="s">
         <v>130</v>
@@ -2832,8 +2835,8 @@
       <c r="C139" s="12">
         <v>2</v>
       </c>
-      <c r="D139" s="15" t="s">
-        <v>145</v>
+      <c r="D139" s="18" t="s">
+        <v>144</v>
       </c>
       <c r="E139" s="16" t="s">
         <v>130</v>
@@ -2846,8 +2849,8 @@
       <c r="C140" s="12">
         <v>2</v>
       </c>
-      <c r="D140" s="18" t="s">
-        <v>146</v>
+      <c r="D140" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="E140" s="16" t="s">
         <v>130</v>
@@ -2860,8 +2863,8 @@
       <c r="C141" s="12">
         <v>2</v>
       </c>
-      <c r="D141" s="15" t="s">
-        <v>147</v>
+      <c r="D141" s="18" t="s">
+        <v>146</v>
       </c>
       <c r="E141" s="16" t="s">
         <v>130</v>
@@ -2874,8 +2877,8 @@
       <c r="C142" s="12">
         <v>2</v>
       </c>
-      <c r="D142" s="18" t="s">
-        <v>148</v>
+      <c r="D142" s="15" t="s">
+        <v>147</v>
       </c>
       <c r="E142" s="16" t="s">
         <v>130</v>
@@ -2888,8 +2891,8 @@
       <c r="C143" s="12">
         <v>2</v>
       </c>
-      <c r="D143" s="15" t="s">
-        <v>149</v>
+      <c r="D143" s="18" t="s">
+        <v>148</v>
       </c>
       <c r="E143" s="16" t="s">
         <v>130</v>
@@ -2900,10 +2903,10 @@
         <v>5</v>
       </c>
       <c r="C144" s="12">
-        <v>6</v>
-      </c>
-      <c r="D144" s="22" t="s">
-        <v>150</v>
+        <v>2</v>
+      </c>
+      <c r="D144" s="15" t="s">
+        <v>149</v>
       </c>
       <c r="E144" s="16" t="s">
         <v>130</v>
@@ -2914,10 +2917,10 @@
         <v>5</v>
       </c>
       <c r="C145" s="12">
-        <v>2</v>
-      </c>
-      <c r="D145" s="15" t="s">
-        <v>151</v>
+        <v>6</v>
+      </c>
+      <c r="D145" s="22" t="s">
+        <v>150</v>
       </c>
       <c r="E145" s="16" t="s">
         <v>130</v>
@@ -2930,8 +2933,8 @@
       <c r="C146" s="12">
         <v>2</v>
       </c>
-      <c r="D146" s="18" t="s">
-        <v>152</v>
+      <c r="D146" s="15" t="s">
+        <v>151</v>
       </c>
       <c r="E146" s="16" t="s">
         <v>130</v>
@@ -2942,10 +2945,10 @@
         <v>5</v>
       </c>
       <c r="C147" s="12">
-        <v>6</v>
-      </c>
-      <c r="D147" s="15" t="s">
-        <v>153</v>
+        <v>2</v>
+      </c>
+      <c r="D147" s="18" t="s">
+        <v>152</v>
       </c>
       <c r="E147" s="16" t="s">
         <v>130</v>
@@ -2958,8 +2961,8 @@
       <c r="C148" s="12">
         <v>6</v>
       </c>
-      <c r="D148" s="18" t="s">
-        <v>154</v>
+      <c r="D148" s="15" t="s">
+        <v>153</v>
       </c>
       <c r="E148" s="16" t="s">
         <v>130</v>
@@ -2972,8 +2975,8 @@
       <c r="C149" s="12">
         <v>6</v>
       </c>
-      <c r="D149" s="15" t="s">
-        <v>155</v>
+      <c r="D149" s="18" t="s">
+        <v>154</v>
       </c>
       <c r="E149" s="16" t="s">
         <v>130</v>
@@ -2986,8 +2989,8 @@
       <c r="C150" s="12">
         <v>6</v>
       </c>
-      <c r="D150" s="22" t="s">
-        <v>156</v>
+      <c r="D150" s="15" t="s">
+        <v>155</v>
       </c>
       <c r="E150" s="16" t="s">
         <v>130</v>
@@ -2998,12 +3001,26 @@
         <v>5</v>
       </c>
       <c r="C151" s="12">
+        <v>6</v>
+      </c>
+      <c r="D151" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="E151" s="16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="152" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B152" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C152" s="12">
         <v>2</v>
       </c>
-      <c r="D151" s="15" t="s">
+      <c r="D152" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="E151" s="16" t="s">
+      <c r="E152" s="16" t="s">
         <v>130</v>
       </c>
     </row>
@@ -3012,10 +3029,10 @@
     <sortCondition ref="D64:D73"/>
   </sortState>
   <mergeCells count="9">
-    <mergeCell ref="B78:E78"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B94:E94"/>
-    <mergeCell ref="B123:E123"/>
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="B90:E90"/>
+    <mergeCell ref="B95:E95"/>
+    <mergeCell ref="B124:E124"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B35:E35"/>
     <mergeCell ref="B15:E15"/>

</xml_diff>

<commit_message>
adding trophy building contest 2
added the trophy for the halloween building contest - 6008
</commit_message>
<xml_diff>
--- a/cmdList.xlsx
+++ b/cmdList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Biamine\ressourcepack\Ressourcepack-for-biamine\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bianca\Desktop\Server biamine\custom plugin\1_Resourcepacks\Github\Ressourcepack-for-biamine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A61182-EDEC-4D2E-9B6C-86B4086486CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F72D77FB-B4F0-48F2-89EA-DD26ECB7F2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Custom Models" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="170">
   <si>
     <t>Key (Legende)</t>
   </si>
@@ -524,6 +524,12 @@
   </si>
   <si>
     <t>trophy: BuildingContest 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - </t>
+  </si>
+  <si>
+    <t>trophy: Building contest 2</t>
   </si>
 </sst>
 </file>
@@ -1065,7 +1071,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J153"/>
+  <dimension ref="B2:J154"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -1315,16 +1321,16 @@
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
-        <v>5</v>
+        <v>168</v>
       </c>
       <c r="C22" s="12">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>30</v>
+        <v>169</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
@@ -1339,10 +1345,10 @@
         <v>7</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
@@ -1357,10 +1363,10 @@
         <v>7</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
@@ -1372,13 +1378,13 @@
         <v>5</v>
       </c>
       <c r="C25" s="12">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
@@ -1393,10 +1399,10 @@
         <v>8</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
@@ -1411,10 +1417,10 @@
         <v>8</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
@@ -1429,10 +1435,10 @@
         <v>8</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
@@ -1447,10 +1453,10 @@
         <v>8</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
@@ -1465,10 +1471,10 @@
         <v>8</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
@@ -1483,10 +1489,10 @@
         <v>8</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
@@ -1498,13 +1504,13 @@
         <v>5</v>
       </c>
       <c r="C32" s="12">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
@@ -1516,13 +1522,13 @@
         <v>5</v>
       </c>
       <c r="C33" s="12">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
@@ -1537,50 +1543,54 @@
         <v>8</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
       <c r="I34" s="8"/>
       <c r="J34" s="4"/>
     </row>
-    <row r="36" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B36" s="23" t="s">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B35" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35" s="12">
+        <v>8</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="4"/>
+    </row>
+    <row r="37" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B37" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="1" t="s">
+      <c r="C37" s="24"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="24"/>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B38" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C38" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D38" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" s="12">
-        <v>6</v>
-      </c>
-      <c r="D38" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
@@ -1591,10 +1601,10 @@
         <v>6</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.25">
@@ -1605,10 +1615,10 @@
         <v>6</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.25">
@@ -1619,10 +1629,10 @@
         <v>6</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.25">
@@ -1633,10 +1643,10 @@
         <v>6</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.25">
@@ -1647,10 +1657,10 @@
         <v>6</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.25">
@@ -1661,10 +1671,10 @@
         <v>6</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.25">
@@ -1675,10 +1685,10 @@
         <v>6</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.25">
@@ -1689,10 +1699,10 @@
         <v>6</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.25">
@@ -1703,10 +1713,10 @@
         <v>6</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.25">
@@ -1717,10 +1727,10 @@
         <v>6</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.25">
@@ -1731,10 +1741,10 @@
         <v>6</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.25">
@@ -1745,10 +1755,10 @@
         <v>6</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.25">
@@ -1759,10 +1769,10 @@
         <v>6</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.25">
@@ -1773,10 +1783,10 @@
         <v>6</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E52" s="14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.25">
@@ -1787,10 +1797,10 @@
         <v>6</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.25">
@@ -1801,10 +1811,10 @@
         <v>6</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.25">
@@ -1815,10 +1825,10 @@
         <v>6</v>
       </c>
       <c r="D55" s="13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.25">
@@ -1829,10 +1839,10 @@
         <v>6</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.25">
@@ -1843,10 +1853,10 @@
         <v>6</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.25">
@@ -1857,10 +1867,10 @@
         <v>6</v>
       </c>
       <c r="D58" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E58" s="14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.25">
@@ -1871,10 +1881,10 @@
         <v>6</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E59" s="14" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.25">
@@ -1885,10 +1895,10 @@
         <v>6</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E60" s="14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.25">
@@ -1899,46 +1909,46 @@
         <v>6</v>
       </c>
       <c r="D61" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="E61" s="14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B62" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62" s="12">
+        <v>6</v>
+      </c>
+      <c r="D62" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E61" s="14" t="s">
+      <c r="E62" s="14" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="63" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B63" s="23" t="s">
+    <row r="64" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B64" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="C63" s="24"/>
-      <c r="D63" s="24"/>
-      <c r="E63" s="24"/>
-    </row>
-    <row r="64" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B64" s="1" t="s">
+      <c r="C64" s="24"/>
+      <c r="D64" s="24"/>
+      <c r="E64" s="24"/>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B65" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C64" s="1" t="s">
+      <c r="C65" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D64" s="1" t="s">
+      <c r="D65" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="E65" s="2" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B65" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C65" s="12">
-        <v>6</v>
-      </c>
-      <c r="D65" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E65" s="14" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
@@ -1949,10 +1959,10 @@
         <v>6</v>
       </c>
       <c r="D66" s="13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E66" s="14" t="s">
-        <v>34</v>
+        <v>161</v>
       </c>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
@@ -1963,10 +1973,10 @@
         <v>6</v>
       </c>
       <c r="D67" s="13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E67" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
@@ -1977,10 +1987,10 @@
         <v>6</v>
       </c>
       <c r="D68" s="13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E68" s="14" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.25">
@@ -1991,10 +2001,10 @@
         <v>6</v>
       </c>
       <c r="D69" s="13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E69" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.25">
@@ -2005,10 +2015,10 @@
         <v>6</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E70" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.25">
@@ -2019,10 +2029,10 @@
         <v>6</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E71" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.25">
@@ -2033,10 +2043,10 @@
         <v>6</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E72" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.25">
@@ -2047,10 +2057,10 @@
         <v>6</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E73" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.25">
@@ -2061,10 +2071,10 @@
         <v>6</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E74" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.25">
@@ -2075,10 +2085,10 @@
         <v>6</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E75" s="14" t="s">
-        <v>163</v>
+        <v>50</v>
       </c>
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.25">
@@ -2089,10 +2099,10 @@
         <v>6</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E76" s="14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.25">
@@ -2103,10 +2113,10 @@
         <v>6</v>
       </c>
       <c r="D77" s="13" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E77" s="14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.25">
@@ -2117,46 +2127,46 @@
         <v>6</v>
       </c>
       <c r="D78" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E78" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B79" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C79" s="12">
+        <v>6</v>
+      </c>
+      <c r="D79" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="E78" s="14" t="s">
+      <c r="E79" s="14" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="80" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B80" s="23" t="s">
+    <row r="81" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B81" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="C80" s="24"/>
-      <c r="D80" s="24"/>
-      <c r="E80" s="24"/>
-    </row>
-    <row r="81" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B81" s="1" t="s">
+      <c r="C81" s="24"/>
+      <c r="D81" s="24"/>
+      <c r="E81" s="24"/>
+    </row>
+    <row r="82" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B82" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C81" s="1" t="s">
+      <c r="C82" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D81" s="1" t="s">
+      <c r="D82" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E81" s="2" t="s">
+      <c r="E82" s="2" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="82" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B82" s="12">
-        <v>1</v>
-      </c>
-      <c r="C82" s="12">
-        <v>1</v>
-      </c>
-      <c r="D82" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E82" s="14" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="83" spans="2:5" x14ac:dyDescent="0.25">
@@ -2167,10 +2177,10 @@
         <v>1</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E83" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="84" spans="2:5" x14ac:dyDescent="0.25">
@@ -2181,10 +2191,10 @@
         <v>1</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E84" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="85" spans="2:5" x14ac:dyDescent="0.25">
@@ -2195,118 +2205,118 @@
         <v>1</v>
       </c>
       <c r="D85" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E85" s="14" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="86" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B86" s="12">
+        <v>1</v>
+      </c>
+      <c r="C86" s="12">
+        <v>1</v>
+      </c>
+      <c r="D86" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E85" s="14" t="s">
+      <c r="E86" s="14" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="89" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B89" s="5"/>
-      <c r="C89" s="7" t="s">
+    <row r="90" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B90" s="5"/>
+      <c r="C90" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="D89" s="5"/>
-      <c r="E89" s="6"/>
-    </row>
-    <row r="91" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B91" s="25" t="s">
+      <c r="D90" s="5"/>
+      <c r="E90" s="6"/>
+    </row>
+    <row r="92" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B92" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="C91" s="24"/>
-      <c r="D91" s="24"/>
-      <c r="E91" s="24"/>
-    </row>
-    <row r="92" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B92" s="1" t="s">
+      <c r="C92" s="24"/>
+      <c r="D92" s="24"/>
+      <c r="E92" s="24"/>
+    </row>
+    <row r="93" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B93" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C92" s="1" t="s">
+      <c r="C93" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D92" s="9" t="s">
+      <c r="D93" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="E92" s="2" t="s">
+      <c r="E93" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="93" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B93" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C93" s="12">
-        <v>6</v>
-      </c>
-      <c r="D93" s="15" t="s">
+    <row r="94" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B94" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C94" s="12">
+        <v>6</v>
+      </c>
+      <c r="D94" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="E93" s="16" t="s">
+      <c r="E94" s="16" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="94" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B94" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="C94" s="17">
-        <v>6</v>
-      </c>
-      <c r="D94" s="18" t="s">
+    <row r="95" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B95" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C95" s="17">
+        <v>6</v>
+      </c>
+      <c r="D95" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="E94" s="19" t="s">
+      <c r="E95" s="19" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="96" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B96" s="25" t="s">
+    <row r="97" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B97" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="C96" s="24"/>
-      <c r="D96" s="24"/>
-      <c r="E96" s="24"/>
-    </row>
-    <row r="97" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B97" s="1" t="s">
+      <c r="C97" s="24"/>
+      <c r="D97" s="24"/>
+      <c r="E97" s="24"/>
+    </row>
+    <row r="98" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B98" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C97" s="1" t="s">
+      <c r="C98" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D97" s="9" t="s">
+      <c r="D98" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="E97" s="2" t="s">
+      <c r="E98" s="2" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="98" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B98" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C98" s="12">
-        <v>6</v>
-      </c>
-      <c r="D98" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E98" s="16" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="99" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B99" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C99" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="D99" s="18" t="s">
-        <v>105</v>
-      </c>
-      <c r="E99" s="21" t="s">
-        <v>104</v>
+      <c r="C99" s="12">
+        <v>6</v>
+      </c>
+      <c r="D99" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="E99" s="16" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="100" spans="2:5" x14ac:dyDescent="0.25">
@@ -2316,8 +2326,8 @@
       <c r="C100" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D100" s="15" t="s">
-        <v>106</v>
+      <c r="D100" s="18" t="s">
+        <v>105</v>
       </c>
       <c r="E100" s="21" t="s">
         <v>104</v>
@@ -2330,8 +2340,8 @@
       <c r="C101" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D101" s="22" t="s">
-        <v>107</v>
+      <c r="D101" s="15" t="s">
+        <v>106</v>
       </c>
       <c r="E101" s="21" t="s">
         <v>104</v>
@@ -2344,8 +2354,8 @@
       <c r="C102" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D102" s="15" t="s">
-        <v>108</v>
+      <c r="D102" s="22" t="s">
+        <v>107</v>
       </c>
       <c r="E102" s="21" t="s">
         <v>104</v>
@@ -2358,8 +2368,8 @@
       <c r="C103" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D103" s="18" t="s">
-        <v>105</v>
+      <c r="D103" s="15" t="s">
+        <v>108</v>
       </c>
       <c r="E103" s="21" t="s">
         <v>104</v>
@@ -2372,8 +2382,8 @@
       <c r="C104" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D104" s="15" t="s">
-        <v>109</v>
+      <c r="D104" s="18" t="s">
+        <v>105</v>
       </c>
       <c r="E104" s="21" t="s">
         <v>104</v>
@@ -2386,8 +2396,8 @@
       <c r="C105" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D105" s="18" t="s">
-        <v>110</v>
+      <c r="D105" s="15" t="s">
+        <v>109</v>
       </c>
       <c r="E105" s="21" t="s">
         <v>104</v>
@@ -2400,8 +2410,8 @@
       <c r="C106" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D106" s="15" t="s">
-        <v>111</v>
+      <c r="D106" s="18" t="s">
+        <v>110</v>
       </c>
       <c r="E106" s="21" t="s">
         <v>104</v>
@@ -2414,8 +2424,8 @@
       <c r="C107" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D107" s="22" t="s">
-        <v>112</v>
+      <c r="D107" s="15" t="s">
+        <v>111</v>
       </c>
       <c r="E107" s="21" t="s">
         <v>104</v>
@@ -2428,8 +2438,8 @@
       <c r="C108" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D108" s="15" t="s">
-        <v>113</v>
+      <c r="D108" s="22" t="s">
+        <v>112</v>
       </c>
       <c r="E108" s="21" t="s">
         <v>104</v>
@@ -2442,8 +2452,8 @@
       <c r="C109" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D109" s="22" t="s">
-        <v>114</v>
+      <c r="D109" s="15" t="s">
+        <v>113</v>
       </c>
       <c r="E109" s="21" t="s">
         <v>104</v>
@@ -2456,8 +2466,8 @@
       <c r="C110" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D110" s="15" t="s">
-        <v>115</v>
+      <c r="D110" s="22" t="s">
+        <v>114</v>
       </c>
       <c r="E110" s="21" t="s">
         <v>104</v>
@@ -2470,8 +2480,8 @@
       <c r="C111" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D111" s="18" t="s">
-        <v>116</v>
+      <c r="D111" s="15" t="s">
+        <v>115</v>
       </c>
       <c r="E111" s="21" t="s">
         <v>104</v>
@@ -2484,8 +2494,8 @@
       <c r="C112" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D112" s="15" t="s">
-        <v>117</v>
+      <c r="D112" s="18" t="s">
+        <v>116</v>
       </c>
       <c r="E112" s="21" t="s">
         <v>104</v>
@@ -2498,8 +2508,8 @@
       <c r="C113" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D113" s="18" t="s">
-        <v>118</v>
+      <c r="D113" s="15" t="s">
+        <v>117</v>
       </c>
       <c r="E113" s="21" t="s">
         <v>104</v>
@@ -2512,8 +2522,8 @@
       <c r="C114" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D114" s="15" t="s">
-        <v>119</v>
+      <c r="D114" s="18" t="s">
+        <v>118</v>
       </c>
       <c r="E114" s="21" t="s">
         <v>104</v>
@@ -2526,8 +2536,8 @@
       <c r="C115" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D115" s="18" t="s">
-        <v>120</v>
+      <c r="D115" s="15" t="s">
+        <v>119</v>
       </c>
       <c r="E115" s="21" t="s">
         <v>104</v>
@@ -2540,8 +2550,8 @@
       <c r="C116" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D116" s="15" t="s">
-        <v>121</v>
+      <c r="D116" s="18" t="s">
+        <v>120</v>
       </c>
       <c r="E116" s="21" t="s">
         <v>104</v>
@@ -2554,8 +2564,8 @@
       <c r="C117" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D117" s="18" t="s">
-        <v>122</v>
+      <c r="D117" s="15" t="s">
+        <v>121</v>
       </c>
       <c r="E117" s="21" t="s">
         <v>104</v>
@@ -2568,8 +2578,8 @@
       <c r="C118" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D118" s="15" t="s">
-        <v>123</v>
+      <c r="D118" s="18" t="s">
+        <v>122</v>
       </c>
       <c r="E118" s="21" t="s">
         <v>104</v>
@@ -2582,8 +2592,8 @@
       <c r="C119" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D119" s="18" t="s">
-        <v>124</v>
+      <c r="D119" s="15" t="s">
+        <v>123</v>
       </c>
       <c r="E119" s="21" t="s">
         <v>104</v>
@@ -2596,8 +2606,8 @@
       <c r="C120" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D120" s="15" t="s">
-        <v>125</v>
+      <c r="D120" s="18" t="s">
+        <v>124</v>
       </c>
       <c r="E120" s="21" t="s">
         <v>104</v>
@@ -2610,8 +2620,8 @@
       <c r="C121" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D121" s="18" t="s">
-        <v>126</v>
+      <c r="D121" s="15" t="s">
+        <v>125</v>
       </c>
       <c r="E121" s="21" t="s">
         <v>104</v>
@@ -2624,8 +2634,8 @@
       <c r="C122" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D122" s="15" t="s">
-        <v>127</v>
+      <c r="D122" s="18" t="s">
+        <v>126</v>
       </c>
       <c r="E122" s="21" t="s">
         <v>104</v>
@@ -2638,47 +2648,47 @@
       <c r="C123" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D123" s="18" t="s">
-        <v>128</v>
+      <c r="D123" s="15" t="s">
+        <v>127</v>
       </c>
       <c r="E123" s="21" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="125" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B125" s="25" t="s">
+    <row r="124" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B124" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C124" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D124" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="E124" s="21" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="126" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B126" s="25" t="s">
         <v>129</v>
       </c>
-      <c r="C125" s="24"/>
-      <c r="D125" s="24"/>
-      <c r="E125" s="24"/>
-    </row>
-    <row r="126" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B126" s="1" t="s">
+      <c r="C126" s="24"/>
+      <c r="D126" s="24"/>
+      <c r="E126" s="24"/>
+    </row>
+    <row r="127" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B127" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C126" s="1" t="s">
+      <c r="C127" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D126" s="9" t="s">
+      <c r="D127" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="E126" s="2" t="s">
+      <c r="E127" s="2" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="127" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B127" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C127" s="12">
-        <v>2</v>
-      </c>
-      <c r="D127" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="E127" s="16" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="128" spans="2:5" x14ac:dyDescent="0.25">
@@ -2688,8 +2698,8 @@
       <c r="C128" s="12">
         <v>2</v>
       </c>
-      <c r="D128" s="18" t="s">
-        <v>132</v>
+      <c r="D128" s="15" t="s">
+        <v>131</v>
       </c>
       <c r="E128" s="16" t="s">
         <v>130</v>
@@ -2702,8 +2712,8 @@
       <c r="C129" s="12">
         <v>2</v>
       </c>
-      <c r="D129" s="15" t="s">
-        <v>133</v>
+      <c r="D129" s="18" t="s">
+        <v>132</v>
       </c>
       <c r="E129" s="16" t="s">
         <v>130</v>
@@ -2716,8 +2726,8 @@
       <c r="C130" s="12">
         <v>2</v>
       </c>
-      <c r="D130" s="22" t="s">
-        <v>134</v>
+      <c r="D130" s="15" t="s">
+        <v>133</v>
       </c>
       <c r="E130" s="16" t="s">
         <v>130</v>
@@ -2730,8 +2740,8 @@
       <c r="C131" s="12">
         <v>2</v>
       </c>
-      <c r="D131" s="15" t="s">
-        <v>135</v>
+      <c r="D131" s="22" t="s">
+        <v>134</v>
       </c>
       <c r="E131" s="16" t="s">
         <v>130</v>
@@ -2744,8 +2754,8 @@
       <c r="C132" s="12">
         <v>2</v>
       </c>
-      <c r="D132" s="18" t="s">
-        <v>136</v>
+      <c r="D132" s="15" t="s">
+        <v>135</v>
       </c>
       <c r="E132" s="16" t="s">
         <v>130</v>
@@ -2758,8 +2768,8 @@
       <c r="C133" s="12">
         <v>2</v>
       </c>
-      <c r="D133" s="15" t="s">
-        <v>137</v>
+      <c r="D133" s="18" t="s">
+        <v>136</v>
       </c>
       <c r="E133" s="16" t="s">
         <v>130</v>
@@ -2772,8 +2782,8 @@
       <c r="C134" s="12">
         <v>2</v>
       </c>
-      <c r="D134" s="22" t="s">
-        <v>138</v>
+      <c r="D134" s="15" t="s">
+        <v>137</v>
       </c>
       <c r="E134" s="16" t="s">
         <v>130</v>
@@ -2786,8 +2796,8 @@
       <c r="C135" s="12">
         <v>2</v>
       </c>
-      <c r="D135" s="15" t="s">
-        <v>139</v>
+      <c r="D135" s="22" t="s">
+        <v>138</v>
       </c>
       <c r="E135" s="16" t="s">
         <v>130</v>
@@ -2800,8 +2810,8 @@
       <c r="C136" s="12">
         <v>2</v>
       </c>
-      <c r="D136" s="22" t="s">
-        <v>140</v>
+      <c r="D136" s="15" t="s">
+        <v>139</v>
       </c>
       <c r="E136" s="16" t="s">
         <v>130</v>
@@ -2814,8 +2824,8 @@
       <c r="C137" s="12">
         <v>2</v>
       </c>
-      <c r="D137" s="15" t="s">
-        <v>141</v>
+      <c r="D137" s="22" t="s">
+        <v>140</v>
       </c>
       <c r="E137" s="16" t="s">
         <v>130</v>
@@ -2828,8 +2838,8 @@
       <c r="C138" s="12">
         <v>2</v>
       </c>
-      <c r="D138" s="22" t="s">
-        <v>142</v>
+      <c r="D138" s="15" t="s">
+        <v>141</v>
       </c>
       <c r="E138" s="16" t="s">
         <v>130</v>
@@ -2842,8 +2852,8 @@
       <c r="C139" s="12">
         <v>2</v>
       </c>
-      <c r="D139" s="15" t="s">
-        <v>143</v>
+      <c r="D139" s="22" t="s">
+        <v>142</v>
       </c>
       <c r="E139" s="16" t="s">
         <v>130</v>
@@ -2856,8 +2866,8 @@
       <c r="C140" s="12">
         <v>2</v>
       </c>
-      <c r="D140" s="18" t="s">
-        <v>144</v>
+      <c r="D140" s="15" t="s">
+        <v>143</v>
       </c>
       <c r="E140" s="16" t="s">
         <v>130</v>
@@ -2870,8 +2880,8 @@
       <c r="C141" s="12">
         <v>2</v>
       </c>
-      <c r="D141" s="15" t="s">
-        <v>145</v>
+      <c r="D141" s="18" t="s">
+        <v>144</v>
       </c>
       <c r="E141" s="16" t="s">
         <v>130</v>
@@ -2884,8 +2894,8 @@
       <c r="C142" s="12">
         <v>2</v>
       </c>
-      <c r="D142" s="18" t="s">
-        <v>146</v>
+      <c r="D142" s="15" t="s">
+        <v>145</v>
       </c>
       <c r="E142" s="16" t="s">
         <v>130</v>
@@ -2898,8 +2908,8 @@
       <c r="C143" s="12">
         <v>2</v>
       </c>
-      <c r="D143" s="15" t="s">
-        <v>147</v>
+      <c r="D143" s="18" t="s">
+        <v>146</v>
       </c>
       <c r="E143" s="16" t="s">
         <v>130</v>
@@ -2912,8 +2922,8 @@
       <c r="C144" s="12">
         <v>2</v>
       </c>
-      <c r="D144" s="18" t="s">
-        <v>148</v>
+      <c r="D144" s="15" t="s">
+        <v>147</v>
       </c>
       <c r="E144" s="16" t="s">
         <v>130</v>
@@ -2926,8 +2936,8 @@
       <c r="C145" s="12">
         <v>2</v>
       </c>
-      <c r="D145" s="15" t="s">
-        <v>149</v>
+      <c r="D145" s="18" t="s">
+        <v>148</v>
       </c>
       <c r="E145" s="16" t="s">
         <v>130</v>
@@ -2938,10 +2948,10 @@
         <v>5</v>
       </c>
       <c r="C146" s="12">
-        <v>6</v>
-      </c>
-      <c r="D146" s="22" t="s">
-        <v>150</v>
+        <v>2</v>
+      </c>
+      <c r="D146" s="15" t="s">
+        <v>149</v>
       </c>
       <c r="E146" s="16" t="s">
         <v>130</v>
@@ -2952,10 +2962,10 @@
         <v>5</v>
       </c>
       <c r="C147" s="12">
-        <v>2</v>
-      </c>
-      <c r="D147" s="15" t="s">
-        <v>151</v>
+        <v>6</v>
+      </c>
+      <c r="D147" s="22" t="s">
+        <v>150</v>
       </c>
       <c r="E147" s="16" t="s">
         <v>130</v>
@@ -2968,8 +2978,8 @@
       <c r="C148" s="12">
         <v>2</v>
       </c>
-      <c r="D148" s="18" t="s">
-        <v>152</v>
+      <c r="D148" s="15" t="s">
+        <v>151</v>
       </c>
       <c r="E148" s="16" t="s">
         <v>130</v>
@@ -2980,10 +2990,10 @@
         <v>5</v>
       </c>
       <c r="C149" s="12">
-        <v>6</v>
-      </c>
-      <c r="D149" s="15" t="s">
-        <v>153</v>
+        <v>2</v>
+      </c>
+      <c r="D149" s="18" t="s">
+        <v>152</v>
       </c>
       <c r="E149" s="16" t="s">
         <v>130</v>
@@ -2996,8 +3006,8 @@
       <c r="C150" s="12">
         <v>6</v>
       </c>
-      <c r="D150" s="18" t="s">
-        <v>154</v>
+      <c r="D150" s="15" t="s">
+        <v>153</v>
       </c>
       <c r="E150" s="16" t="s">
         <v>130</v>
@@ -3010,8 +3020,8 @@
       <c r="C151" s="12">
         <v>6</v>
       </c>
-      <c r="D151" s="15" t="s">
-        <v>155</v>
+      <c r="D151" s="18" t="s">
+        <v>154</v>
       </c>
       <c r="E151" s="16" t="s">
         <v>130</v>
@@ -3024,8 +3034,8 @@
       <c r="C152" s="12">
         <v>6</v>
       </c>
-      <c r="D152" s="22" t="s">
-        <v>156</v>
+      <c r="D152" s="15" t="s">
+        <v>155</v>
       </c>
       <c r="E152" s="16" t="s">
         <v>130</v>
@@ -3036,29 +3046,43 @@
         <v>5</v>
       </c>
       <c r="C153" s="12">
-        <v>2</v>
-      </c>
-      <c r="D153" s="15" t="s">
-        <v>157</v>
+        <v>6</v>
+      </c>
+      <c r="D153" s="22" t="s">
+        <v>156</v>
       </c>
       <c r="E153" s="16" t="s">
         <v>130</v>
       </c>
     </row>
+    <row r="154" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B154" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C154" s="12">
+        <v>2</v>
+      </c>
+      <c r="D154" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="E154" s="16" t="s">
+        <v>130</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B65:E74">
-    <sortCondition ref="D65:D74"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B66:E75">
+    <sortCondition ref="D66:D75"/>
   </sortState>
   <mergeCells count="9">
-    <mergeCell ref="B80:E80"/>
-    <mergeCell ref="B91:E91"/>
-    <mergeCell ref="B96:E96"/>
-    <mergeCell ref="B125:E125"/>
+    <mergeCell ref="B81:E81"/>
+    <mergeCell ref="B92:E92"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="B126:E126"/>
     <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B37:E37"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B64:E64"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>